<commit_message>
Wipe survey data and add /reset command
</commit_message>
<xml_diff>
--- a/survey_results.xlsx
+++ b/survey_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -443,31 +443,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2026-08-25 23:56:04</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>1537845176</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>𝖙𝖊𝖘𝖋𝖆</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>@Shetesfa</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>1. በነበረው ይቀጥል (09:00 - 11:00)</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>